<commit_message>
Update leave parental home process
</commit_message>
<xml_diff>
--- a/input/reg_leaveParentalHome.xlsx
+++ b/input/reg_leaveParentalHome.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patryk\git\SimPaths_HU\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59318DA2-7DDB-4CA0-84C7-6F53D92EB71B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF267F57-0036-4059-BFD5-C8703053DA5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
-    <sheet name="IT_P1a" sheetId="3" r:id="rId2"/>
+    <sheet name="EL_P1a" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="25">
   <si>
     <t>Description:</t>
   </si>
@@ -89,19 +89,13 @@
     <t>Constant</t>
   </si>
   <si>
-    <t>Regions: ITF = South, ITG = Islands, ITH = Northeast, ITI = Central. Northwest (ITC) is the omitted region.</t>
-  </si>
-  <si>
-    <t>ITF</t>
-  </si>
-  <si>
-    <t>ITG</t>
-  </si>
-  <si>
-    <t>ITH</t>
-  </si>
-  <si>
-    <t>ITI</t>
+    <t>Regions: EL3 = Attika (omitted), EL4 = Aegean Islands, EL7 = Central and Northern Greece</t>
+  </si>
+  <si>
+    <t>EL4</t>
+  </si>
+  <si>
+    <t>EL7</t>
   </si>
 </sst>
 </file>
@@ -484,9 +478,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -494,7 +488,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -502,7 +496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -510,7 +504,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
@@ -525,13 +519,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:T19"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:R17"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.86328125" customWidth="1"/>
+    <col min="1" max="1" width="21.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -578,1135 +572,909 @@
         <v>24</v>
       </c>
       <c r="P1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="Q1" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="R1" t="s">
-        <v>19</v>
-      </c>
-      <c r="S1" t="s">
-        <v>20</v>
-      </c>
-      <c r="T1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
       <c r="B2">
-        <v>-0.11665255243619094</v>
+        <v>-0.11393604583496905</v>
       </c>
       <c r="C2">
-        <v>3.1072053774141048E-3</v>
+        <v>7.7489549560344336E-3</v>
       </c>
       <c r="D2">
-        <v>5.3018779782759603E-5</v>
+        <v>-2.8215442766438926E-4</v>
       </c>
       <c r="E2">
-        <v>-3.8824340580041835E-7</v>
+        <v>3.2735681758690441E-6</v>
       </c>
       <c r="F2">
-        <v>1.9971902367906674E-4</v>
+        <v>-1.5347609326089836E-3</v>
       </c>
       <c r="G2">
-        <v>2.1342907149638491E-4</v>
+        <v>-2.6511799641848362E-3</v>
       </c>
       <c r="H2">
-        <v>6.5297588585840299E-4</v>
+        <v>2.7377980390724073E-3</v>
       </c>
       <c r="I2">
-        <v>2.7761284365612169E-4</v>
+        <v>1.2909561662087755E-3</v>
       </c>
       <c r="J2">
-        <v>1.9996577603494675E-4</v>
+        <v>1.1716383936679828E-3</v>
       </c>
       <c r="K2">
-        <v>2.9751552969763015E-4</v>
+        <v>6.6050970486672097E-4</v>
       </c>
       <c r="L2">
-        <v>-2.9177979542105101E-4</v>
+        <v>-7.0038899934689812E-4</v>
       </c>
       <c r="M2">
-        <v>2.1171902245266101E-4</v>
+        <v>-7.797239069494582E-4</v>
       </c>
       <c r="N2">
-        <v>1.6792533159027054E-4</v>
+        <v>-3.1516198267035871E-4</v>
       </c>
       <c r="O2">
-        <v>-6.6383971844634077E-4</v>
+        <v>-1.4751464401400835E-3</v>
       </c>
       <c r="P2">
-        <v>1.4827892130014485E-4</v>
+        <v>-1.0836520001444264E-4</v>
       </c>
       <c r="Q2">
-        <v>-9.5053186783118391E-5</v>
+        <v>-3.3466507370939758E-4</v>
       </c>
       <c r="R2">
-        <v>-7.7364248326043373E-6</v>
-      </c>
-      <c r="S2">
-        <v>-6.5627161746209279E-4</v>
-      </c>
-      <c r="T2">
-        <v>-3.3823911252607811E-3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.45">
+        <v>4.7173049938376722E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
       <c r="B3">
-        <v>1.5959002028928627E-2</v>
+        <v>3.8482211591740756E-2</v>
       </c>
       <c r="C3">
-        <v>5.3018779782759603E-5</v>
+        <v>-2.8215442766438926E-4</v>
       </c>
       <c r="D3">
-        <v>1.9540707253068695E-4</v>
+        <v>4.4450884815583217E-4</v>
       </c>
       <c r="E3">
-        <v>-2.0384986038459955E-6</v>
+        <v>-4.7772235768318784E-6</v>
       </c>
       <c r="F3">
-        <v>-1.0346847977282412E-5</v>
+        <v>3.063953637296845E-4</v>
       </c>
       <c r="G3">
-        <v>-1.1762252871309431E-4</v>
+        <v>2.1407622493884587E-4</v>
       </c>
       <c r="H3">
-        <v>8.2841807353551419E-4</v>
+        <v>1.4834346174939046E-3</v>
       </c>
       <c r="I3">
-        <v>1.0388297784687966E-4</v>
+        <v>-4.5246932897106528E-4</v>
       </c>
       <c r="J3">
-        <v>1.0366338802755934E-4</v>
+        <v>1.7874113095826247E-4</v>
       </c>
       <c r="K3">
-        <v>2.0805397281212831E-4</v>
+        <v>-3.5551982551349295E-4</v>
       </c>
       <c r="L3">
-        <v>-1.1055136486285214E-5</v>
+        <v>-3.677064740092266E-4</v>
       </c>
       <c r="M3">
-        <v>-9.2400379162897988E-5</v>
+        <v>3.7845676564568151E-5</v>
       </c>
       <c r="N3">
-        <v>-1.3884152318324261E-4</v>
+        <v>-5.5699058760231082E-4</v>
       </c>
       <c r="O3">
-        <v>-2.6588169724675652E-4</v>
+        <v>-3.0856500019985425E-4</v>
       </c>
       <c r="P3">
-        <v>-1.7171163662585268E-4</v>
+        <v>2.0146364281990227E-5</v>
       </c>
       <c r="Q3">
-        <v>-2.6502242576178798E-4</v>
+        <v>1.3248957791701862E-3</v>
       </c>
       <c r="R3">
-        <v>-8.9100406146334498E-6</v>
-      </c>
-      <c r="S3">
-        <v>-2.7610964267736214E-4</v>
-      </c>
-      <c r="T3">
-        <v>-4.0679282969788861E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.45">
+        <v>-9.6179073198524243E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
       <c r="B4">
-        <v>2.9471462899883236E-4</v>
+        <v>1.3469942057824357E-4</v>
       </c>
       <c r="C4">
-        <v>-3.8824340580041835E-7</v>
+        <v>3.2735681758690441E-6</v>
       </c>
       <c r="D4">
-        <v>-2.0384986038459955E-6</v>
+        <v>-4.7772235768318784E-6</v>
       </c>
       <c r="E4">
-        <v>2.1896228208100444E-8</v>
+        <v>5.2347312925267616E-8</v>
       </c>
       <c r="F4">
-        <v>5.7084788703991417E-7</v>
+        <v>-3.5316569938889295E-6</v>
       </c>
       <c r="G4">
-        <v>1.316578382667805E-6</v>
+        <v>-2.8814730291068801E-6</v>
       </c>
       <c r="H4">
-        <v>-7.6566532169463463E-6</v>
+        <v>-1.4843144331407232E-5</v>
       </c>
       <c r="I4">
-        <v>-1.3067959153437273E-6</v>
+        <v>4.1138833152178749E-6</v>
       </c>
       <c r="J4">
-        <v>-7.9670026895101053E-7</v>
+        <v>-2.6245668130097566E-6</v>
       </c>
       <c r="K4">
-        <v>-1.6205127887724578E-6</v>
+        <v>3.2449317574659401E-6</v>
       </c>
       <c r="L4">
-        <v>3.7445727839454096E-7</v>
+        <v>3.3798366878817511E-6</v>
       </c>
       <c r="M4">
-        <v>1.1793410995312413E-6</v>
+        <v>-1.1135470244832068E-6</v>
       </c>
       <c r="N4">
-        <v>1.8024596597384412E-6</v>
+        <v>6.5681275104355146E-6</v>
       </c>
       <c r="O4">
-        <v>2.8894378140545946E-6</v>
+        <v>3.3824982748285859E-6</v>
       </c>
       <c r="P4">
-        <v>1.5359142673637339E-6</v>
+        <v>-2.1259597245707897E-7</v>
       </c>
       <c r="Q4">
-        <v>2.438407671292133E-6</v>
+        <v>-1.396862500921772E-5</v>
       </c>
       <c r="R4">
-        <v>4.0657622425960691E-8</v>
-      </c>
-      <c r="S4">
-        <v>2.809613806166921E-6</v>
-      </c>
-      <c r="T4">
-        <v>4.1336281359242754E-5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.45">
+        <v>1.019425455645008E-4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
       <c r="B5">
-        <v>8.4153018387571471E-2</v>
+        <v>0.29528297997668695</v>
       </c>
       <c r="C5">
-        <v>1.9971902367906674E-4</v>
+        <v>-1.5347609326089836E-3</v>
       </c>
       <c r="D5">
-        <v>-1.0346847977282412E-5</v>
+        <v>3.063953637296845E-4</v>
       </c>
       <c r="E5">
-        <v>5.7084788703991417E-7</v>
+        <v>-3.5316569938889295E-6</v>
       </c>
       <c r="F5">
-        <v>7.5342832814023807E-3</v>
+        <v>1.1643306771341531E-2</v>
       </c>
       <c r="G5">
-        <v>5.8743758350544382E-3</v>
+        <v>9.4658182134819274E-3</v>
       </c>
       <c r="H5">
-        <v>3.9301068216984368E-4</v>
+        <v>-1.9674634300151103E-3</v>
       </c>
       <c r="I5">
-        <v>-8.147106009014657E-4</v>
+        <v>-8.3568878316672571E-4</v>
       </c>
       <c r="J5">
-        <v>1.8619441540778355E-3</v>
+        <v>-2.9031770789665354E-3</v>
       </c>
       <c r="K5">
-        <v>1.3965063238404558E-3</v>
+        <v>3.7244393780023924E-4</v>
       </c>
       <c r="L5">
-        <v>1.5513213744295208E-3</v>
+        <v>-1.5993801741075208E-3</v>
       </c>
       <c r="M5">
-        <v>2.8476683861385728E-3</v>
+        <v>4.6356856804825484E-3</v>
       </c>
       <c r="N5">
-        <v>1.2628516551870098E-3</v>
+        <v>-4.6855425217653696E-3</v>
       </c>
       <c r="O5">
-        <v>1.7452778991200975E-3</v>
+        <v>-4.0870362733583226E-3</v>
       </c>
       <c r="P5">
-        <v>2.2592037170349449E-4</v>
+        <v>-1.0061650106994697E-4</v>
       </c>
       <c r="Q5">
-        <v>-2.4121382828014358E-4</v>
+        <v>1.1107556451979448E-2</v>
       </c>
       <c r="R5">
-        <v>-1.8265244248629289E-4</v>
-      </c>
-      <c r="S5">
-        <v>9.9638628181522083E-4</v>
-      </c>
-      <c r="T5">
-        <v>-5.3423360247093279E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.45">
+        <v>-1.0361329999183677E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
       <c r="B6">
-        <v>5.2612775087819218E-2</v>
+        <v>0.33522745536722492</v>
       </c>
       <c r="C6">
-        <v>2.1342907149638491E-4</v>
+        <v>-2.6511799641848362E-3</v>
       </c>
       <c r="D6">
-        <v>-1.1762252871309431E-4</v>
+        <v>2.1407622493884587E-4</v>
       </c>
       <c r="E6">
-        <v>1.316578382667805E-6</v>
+        <v>-2.8814730291068801E-6</v>
       </c>
       <c r="F6">
-        <v>5.8743758350544382E-3</v>
+        <v>9.4658182134819274E-3</v>
       </c>
       <c r="G6">
-        <v>8.4708141667496767E-3</v>
+        <v>1.2760348948721176E-2</v>
       </c>
       <c r="H6">
-        <v>-2.7288204424195939E-4</v>
+        <v>-1.3264958638944434E-3</v>
       </c>
       <c r="I6">
-        <v>-1.8447962727405035E-3</v>
+        <v>-1.4265385680514706E-3</v>
       </c>
       <c r="J6">
-        <v>2.2307637882138564E-3</v>
+        <v>-3.007624038211568E-3</v>
       </c>
       <c r="K6">
-        <v>1.4104440563031469E-3</v>
+        <v>4.3046781176135087E-4</v>
       </c>
       <c r="L6">
-        <v>1.1936431935963047E-3</v>
+        <v>-2.9237219077708933E-4</v>
       </c>
       <c r="M6">
-        <v>3.4099513425915121E-3</v>
+        <v>4.2930882624070809E-3</v>
       </c>
       <c r="N6">
-        <v>1.6574776638180989E-3</v>
+        <v>-3.7078885158066538E-3</v>
       </c>
       <c r="O6">
-        <v>9.495491834324403E-4</v>
+        <v>-2.5905462388995824E-3</v>
       </c>
       <c r="P6">
-        <v>1.2379578923736121E-3</v>
+        <v>-5.5516971335677908E-5</v>
       </c>
       <c r="Q6">
-        <v>4.4738993930741003E-4</v>
+        <v>8.8369813352681039E-3</v>
       </c>
       <c r="R6">
-        <v>-1.2569327006975626E-4</v>
-      </c>
-      <c r="S6">
-        <v>1.6293921218012769E-3</v>
-      </c>
-      <c r="T6">
-        <v>-3.364111670384847E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.45">
+        <v>-8.1509555860503971E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
       <c r="B7">
-        <v>-0.37650018517925599</v>
+        <v>0.15909748149908723</v>
       </c>
       <c r="C7">
-        <v>6.5297588585840299E-4</v>
+        <v>2.7377980390724073E-3</v>
       </c>
       <c r="D7">
-        <v>8.2841807353551419E-4</v>
+        <v>1.4834346174939046E-3</v>
       </c>
       <c r="E7">
-        <v>-7.6566532169463463E-6</v>
+        <v>-1.4843144331407232E-5</v>
       </c>
       <c r="F7">
-        <v>3.9301068216984368E-4</v>
+        <v>-1.9674634300151103E-3</v>
       </c>
       <c r="G7">
-        <v>-2.7288204424195939E-4</v>
+        <v>-1.3264958638944434E-3</v>
       </c>
       <c r="H7">
-        <v>3.4123409077127728E-2</v>
+        <v>4.8860315108496866E-2</v>
       </c>
       <c r="I7">
-        <v>5.5415939115344443E-3</v>
+        <v>3.1876840016164662E-3</v>
       </c>
       <c r="J7">
-        <v>1.4807351369124221E-3</v>
+        <v>-5.5637697395646479E-3</v>
       </c>
       <c r="K7">
-        <v>5.2732422650741129E-3</v>
+        <v>-5.0551596664057969E-3</v>
       </c>
       <c r="L7">
-        <v>7.105257148090822E-3</v>
+        <v>5.069226035869373E-4</v>
       </c>
       <c r="M7">
-        <v>7.4877982395360997E-3</v>
+        <v>-6.52298430825482E-4</v>
       </c>
       <c r="N7">
-        <v>-1.0158582408914974E-4</v>
+        <v>-3.2564127191624104E-4</v>
       </c>
       <c r="O7">
-        <v>-1.9493040940848092E-3</v>
+        <v>-2.9163271951140879E-5</v>
       </c>
       <c r="P7">
-        <v>-1.6653665831099914E-3</v>
+        <v>4.5171837507327608E-4</v>
       </c>
       <c r="Q7">
-        <v>-2.5592008068141183E-3</v>
+        <v>-1.2415343685808766E-3</v>
       </c>
       <c r="R7">
-        <v>-2.0138015442662744E-4</v>
-      </c>
-      <c r="S7">
-        <v>-2.2488595407094917E-3</v>
-      </c>
-      <c r="T7">
-        <v>-2.3850308120631505E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.45">
+        <v>-4.3199896539518431E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
       <c r="B8">
-        <v>-0.10710973726362788</v>
+        <v>-7.8941547075418325E-2</v>
       </c>
       <c r="C8">
-        <v>2.7761284365612169E-4</v>
+        <v>1.2909561662087755E-3</v>
       </c>
       <c r="D8">
-        <v>1.0388297784687966E-4</v>
+        <v>-4.5246932897106528E-4</v>
       </c>
       <c r="E8">
-        <v>-1.3067959153437273E-6</v>
+        <v>4.1138833152178749E-6</v>
       </c>
       <c r="F8">
-        <v>-8.147106009014657E-4</v>
+        <v>-8.3568878316672571E-4</v>
       </c>
       <c r="G8">
-        <v>-1.8447962727405035E-3</v>
+        <v>-1.4265385680514706E-3</v>
       </c>
       <c r="H8">
-        <v>5.5415939115344443E-3</v>
+        <v>3.1876840016164662E-3</v>
       </c>
       <c r="I8">
-        <v>7.4316845415800803E-3</v>
+        <v>1.1167540337020922E-2</v>
       </c>
       <c r="J8">
-        <v>5.3784358319891633E-5</v>
+        <v>1.2596638396637481E-3</v>
       </c>
       <c r="K8">
-        <v>3.1873406689018808E-3</v>
+        <v>5.8052617617816342E-3</v>
       </c>
       <c r="L8">
-        <v>5.3080861455184298E-3</v>
+        <v>9.2928091246304786E-3</v>
       </c>
       <c r="M8">
-        <v>6.0771010436227613E-3</v>
+        <v>9.0823053083061538E-3</v>
       </c>
       <c r="N8">
-        <v>-5.2892941473478474E-4</v>
+        <v>5.8211774263378785E-4</v>
       </c>
       <c r="O8">
-        <v>2.8042670290388588E-4</v>
+        <v>6.0372941565419239E-4</v>
       </c>
       <c r="P8">
-        <v>-1.4460380100188514E-4</v>
+        <v>-1.2967331318152614E-5</v>
       </c>
       <c r="Q8">
-        <v>-8.3485450364707879E-5</v>
+        <v>-1.8771328538540744E-3</v>
       </c>
       <c r="R8">
-        <v>1.1475949648633461E-4</v>
-      </c>
-      <c r="S8">
-        <v>-1.2760094487212347E-3</v>
-      </c>
-      <c r="T8">
-        <v>-8.592742683163344E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.45">
+        <v>9.5786317840187984E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
       <c r="B9">
-        <v>3.5769616167039116E-2</v>
+        <v>-0.18103540029735291</v>
       </c>
       <c r="C9">
-        <v>1.9996577603494675E-4</v>
+        <v>1.1716383936679828E-3</v>
       </c>
       <c r="D9">
-        <v>1.0366338802755934E-4</v>
+        <v>1.7874113095826247E-4</v>
       </c>
       <c r="E9">
-        <v>-7.9670026895101053E-7</v>
+        <v>-2.6245668130097566E-6</v>
       </c>
       <c r="F9">
-        <v>1.8619441540778355E-3</v>
+        <v>-2.9031770789665354E-3</v>
       </c>
       <c r="G9">
-        <v>2.2307637882138564E-3</v>
+        <v>-3.007624038211568E-3</v>
       </c>
       <c r="H9">
-        <v>1.4807351369124221E-3</v>
+        <v>-5.5637697395646479E-3</v>
       </c>
       <c r="I9">
-        <v>5.3784358319891633E-5</v>
+        <v>1.2596638396637481E-3</v>
       </c>
       <c r="J9">
-        <v>9.3100487869486933E-3</v>
+        <v>1.2722713423747999E-2</v>
       </c>
       <c r="K9">
-        <v>5.6929248491320505E-3</v>
+        <v>4.7472628194184224E-3</v>
       </c>
       <c r="L9">
-        <v>5.7130556620046836E-3</v>
+        <v>4.9629549329938448E-3</v>
       </c>
       <c r="M9">
-        <v>5.9944636699121945E-3</v>
+        <v>3.8748416232493293E-3</v>
       </c>
       <c r="N9">
-        <v>4.1844943811320456E-4</v>
+        <v>-1.1001440045025259E-3</v>
       </c>
       <c r="O9">
-        <v>1.5531217400553126E-3</v>
+        <v>-5.8893333344320342E-4</v>
       </c>
       <c r="P9">
-        <v>5.1974690662834853E-5</v>
+        <v>-4.2537009316695543E-5</v>
       </c>
       <c r="Q9">
-        <v>-9.7095857401441809E-4</v>
+        <v>-5.0012867754745984E-4</v>
       </c>
       <c r="R9">
-        <v>-1.796116370937893E-4</v>
-      </c>
-      <c r="S9">
-        <v>7.701805963137155E-4</v>
-      </c>
-      <c r="T9">
-        <v>-7.3773887527030114E-3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.45">
+        <v>-4.5658547075397883E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>16</v>
       </c>
       <c r="B10">
-        <v>3.8106229585599352E-2</v>
+        <v>0.15800130562840087</v>
       </c>
       <c r="C10">
-        <v>2.9751552969763015E-4</v>
+        <v>6.6050970486672097E-4</v>
       </c>
       <c r="D10">
-        <v>2.0805397281212831E-4</v>
+        <v>-3.5551982551349295E-4</v>
       </c>
       <c r="E10">
-        <v>-1.6205127887724578E-6</v>
+        <v>3.2449317574659401E-6</v>
       </c>
       <c r="F10">
-        <v>1.3965063238404558E-3</v>
+        <v>3.7244393780023924E-4</v>
       </c>
       <c r="G10">
-        <v>1.4104440563031469E-3</v>
+        <v>4.3046781176135087E-4</v>
       </c>
       <c r="H10">
-        <v>5.2732422650741129E-3</v>
+        <v>-5.0551596664057969E-3</v>
       </c>
       <c r="I10">
-        <v>3.1873406689018808E-3</v>
+        <v>5.8052617617816342E-3</v>
       </c>
       <c r="J10">
-        <v>5.6929248491320505E-3</v>
+        <v>4.7472628194184224E-3</v>
       </c>
       <c r="K10">
-        <v>1.0549208267044087E-2</v>
+        <v>1.2925971515695635E-2</v>
       </c>
       <c r="L10">
-        <v>8.2866188271756205E-3</v>
+        <v>9.3444641604198617E-3</v>
       </c>
       <c r="M10">
-        <v>9.0756886692523638E-3</v>
+        <v>9.9358240094997701E-3</v>
       </c>
       <c r="N10">
-        <v>4.7405251752729227E-4</v>
+        <v>-9.5082125552503616E-4</v>
       </c>
       <c r="O10">
-        <v>2.1661542361902462E-3</v>
+        <v>-7.3377462973899486E-4</v>
       </c>
       <c r="P10">
-        <v>-2.0619608947031838E-4</v>
+        <v>-2.044245098543395E-4</v>
       </c>
       <c r="Q10">
-        <v>-1.1966821541551983E-3</v>
+        <v>7.7797411614440037E-4</v>
       </c>
       <c r="R10">
-        <v>-1.9558995899237713E-4</v>
-      </c>
-      <c r="S10">
-        <v>4.1501640030809249E-4</v>
-      </c>
-      <c r="T10">
-        <v>-1.241450547843256E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.45">
+        <v>2.1790331888380116E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>17</v>
       </c>
       <c r="B11">
-        <v>1.8820203111344021E-2</v>
+        <v>-2.7655616126871854E-2</v>
       </c>
       <c r="C11">
-        <v>-2.9177979542105101E-4</v>
+        <v>-7.0038899934689812E-4</v>
       </c>
       <c r="D11">
-        <v>-1.1055136486285214E-5</v>
+        <v>-3.677064740092266E-4</v>
       </c>
       <c r="E11">
-        <v>3.7445727839454096E-7</v>
+        <v>3.3798366878817511E-6</v>
       </c>
       <c r="F11">
-        <v>1.5513213744295208E-3</v>
+        <v>-1.5993801741075208E-3</v>
       </c>
       <c r="G11">
-        <v>1.1936431935963047E-3</v>
+        <v>-2.9237219077708933E-4</v>
       </c>
       <c r="H11">
-        <v>7.105257148090822E-3</v>
+        <v>5.069226035869373E-4</v>
       </c>
       <c r="I11">
-        <v>5.3080861455184298E-3</v>
+        <v>9.2928091246304786E-3</v>
       </c>
       <c r="J11">
-        <v>5.7130556620046836E-3</v>
+        <v>4.9629549329938448E-3</v>
       </c>
       <c r="K11">
-        <v>8.2866188271756205E-3</v>
+        <v>9.3444641604198617E-3</v>
       </c>
       <c r="L11">
-        <v>1.3578480439716659E-2</v>
+        <v>1.733589474764894E-2</v>
       </c>
       <c r="M11">
-        <v>1.1400266877747405E-2</v>
+        <v>1.2333668584484446E-2</v>
       </c>
       <c r="N11">
-        <v>6.4350485594438442E-4</v>
+        <v>2.4028295164946201E-4</v>
       </c>
       <c r="O11">
-        <v>3.332664544750548E-3</v>
+        <v>1.5327164508533719E-3</v>
       </c>
       <c r="P11">
-        <v>-5.3155510186194484E-4</v>
+        <v>-4.7491405347423687E-5</v>
       </c>
       <c r="Q11">
-        <v>-1.3963484469953419E-3</v>
+        <v>-2.3568185003525477E-3</v>
       </c>
       <c r="R11">
-        <v>-7.175216639173981E-5</v>
-      </c>
-      <c r="S11">
-        <v>9.0241584827686992E-4</v>
-      </c>
-      <c r="T11">
-        <v>-1.0816096040140584E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.45">
+        <v>-2.6313988096598809E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
       </c>
       <c r="B12">
-        <v>-0.20729245419238287</v>
+        <v>0.19538918029121674</v>
       </c>
       <c r="C12">
-        <v>2.1171902245266101E-4</v>
+        <v>-7.797239069494582E-4</v>
       </c>
       <c r="D12">
-        <v>-9.2400379162897988E-5</v>
+        <v>3.7845676564568151E-5</v>
       </c>
       <c r="E12">
-        <v>1.1793410995312413E-6</v>
+        <v>-1.1135470244832068E-6</v>
       </c>
       <c r="F12">
-        <v>2.8476683861385728E-3</v>
+        <v>4.6356856804825484E-3</v>
       </c>
       <c r="G12">
-        <v>3.4099513425915121E-3</v>
+        <v>4.2930882624070809E-3</v>
       </c>
       <c r="H12">
-        <v>7.4877982395360997E-3</v>
+        <v>-6.52298430825482E-4</v>
       </c>
       <c r="I12">
-        <v>6.0771010436227613E-3</v>
+        <v>9.0823053083061538E-3</v>
       </c>
       <c r="J12">
-        <v>5.9944636699121945E-3</v>
+        <v>3.8748416232493293E-3</v>
       </c>
       <c r="K12">
-        <v>9.0756886692523638E-3</v>
+        <v>9.9358240094997701E-3</v>
       </c>
       <c r="L12">
-        <v>1.1400266877747405E-2</v>
+        <v>1.2333668584484446E-2</v>
       </c>
       <c r="M12">
-        <v>1.7445742320793219E-2</v>
+        <v>2.043503819425033E-2</v>
       </c>
       <c r="N12">
-        <v>1.4287844362998849E-3</v>
+        <v>-5.1735723901076211E-3</v>
       </c>
       <c r="O12">
-        <v>3.0681753543927901E-3</v>
+        <v>-3.2199563110128435E-3</v>
       </c>
       <c r="P12">
-        <v>-7.546836858702481E-5</v>
+        <v>-1.108460694897777E-4</v>
       </c>
       <c r="Q12">
-        <v>1.82046751185376E-4</v>
+        <v>1.042019450191789E-2</v>
       </c>
       <c r="R12">
-        <v>-5.8933168319049995E-5</v>
-      </c>
-      <c r="S12">
-        <v>2.0450145324684473E-4</v>
-      </c>
-      <c r="T12">
-        <v>-1.2345642577996694E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.45">
+        <v>-1.3117976257928422E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>23</v>
       </c>
       <c r="B13">
-        <v>-0.21137282477383562</v>
+        <v>-0.44051975834799939</v>
       </c>
       <c r="C13">
-        <v>1.6792533159027054E-4</v>
+        <v>-3.1516198267035871E-4</v>
       </c>
       <c r="D13">
-        <v>-1.3884152318324261E-4</v>
+        <v>-5.5699058760231082E-4</v>
       </c>
       <c r="E13">
-        <v>1.8024596597384412E-6</v>
+        <v>6.5681275104355146E-6</v>
       </c>
       <c r="F13">
-        <v>1.2628516551870098E-3</v>
+        <v>-4.6855425217653696E-3</v>
       </c>
       <c r="G13">
-        <v>1.6574776638180989E-3</v>
+        <v>-3.7078885158066538E-3</v>
       </c>
       <c r="H13">
-        <v>-1.0158582408914974E-4</v>
+        <v>-3.2564127191624104E-4</v>
       </c>
       <c r="I13">
-        <v>-5.2892941473478474E-4</v>
+        <v>5.8211774263378785E-4</v>
       </c>
       <c r="J13">
-        <v>4.1844943811320456E-4</v>
+        <v>-1.1001440045025259E-3</v>
       </c>
       <c r="K13">
-        <v>4.7405251752729227E-4</v>
+        <v>-9.5082125552503616E-4</v>
       </c>
       <c r="L13">
-        <v>6.4350485594438442E-4</v>
+        <v>2.4028295164946201E-4</v>
       </c>
       <c r="M13">
-        <v>1.4287844362998849E-3</v>
+        <v>-5.1735723901076211E-3</v>
       </c>
       <c r="N13">
-        <v>6.8279757914291462E-3</v>
+        <v>1.5176393094593857E-2</v>
       </c>
       <c r="O13">
-        <v>3.8230087420125405E-3</v>
+        <v>6.0785809689776118E-3</v>
       </c>
       <c r="P13">
-        <v>3.0587759543058723E-3</v>
+        <v>2.1641988894057277E-5</v>
       </c>
       <c r="Q13">
-        <v>3.2389422085004355E-3</v>
+        <v>-1.0732736406725899E-2</v>
       </c>
       <c r="R13">
-        <v>-1.342885853051428E-4</v>
-      </c>
-      <c r="S13">
-        <v>8.6147130719185197E-4</v>
-      </c>
-      <c r="T13">
-        <v>-5.4344618842005609E-4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.45">
+        <v>1.1057574606980491E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>24</v>
       </c>
       <c r="B14">
-        <v>-6.5470798314513967E-2</v>
+        <v>-0.30777237429387388</v>
       </c>
       <c r="C14">
-        <v>-6.6383971844634077E-4</v>
+        <v>-1.4751464401400835E-3</v>
       </c>
       <c r="D14">
-        <v>-2.6588169724675652E-4</v>
+        <v>-3.0856500019985425E-4</v>
       </c>
       <c r="E14">
-        <v>2.8894378140545946E-6</v>
+        <v>3.3824982748285859E-6</v>
       </c>
       <c r="F14">
-        <v>1.7452778991200975E-3</v>
+        <v>-4.0870362733583226E-3</v>
       </c>
       <c r="G14">
-        <v>9.495491834324403E-4</v>
+        <v>-2.5905462388995824E-3</v>
       </c>
       <c r="H14">
-        <v>-1.9493040940848092E-3</v>
+        <v>-2.9163271951140879E-5</v>
       </c>
       <c r="I14">
-        <v>2.8042670290388588E-4</v>
+        <v>6.0372941565419239E-4</v>
       </c>
       <c r="J14">
-        <v>1.5531217400553126E-3</v>
+        <v>-5.8893333344320342E-4</v>
       </c>
       <c r="K14">
-        <v>2.1661542361902462E-3</v>
+        <v>-7.3377462973899486E-4</v>
       </c>
       <c r="L14">
-        <v>3.332664544750548E-3</v>
+        <v>1.5327164508533719E-3</v>
       </c>
       <c r="M14">
-        <v>3.0681753543927901E-3</v>
+        <v>-3.2199563110128435E-3</v>
       </c>
       <c r="N14">
-        <v>3.8230087420125405E-3</v>
+        <v>6.0785809689776118E-3</v>
       </c>
       <c r="O14">
-        <v>1.2431552252368812E-2</v>
+        <v>7.5764183133913837E-3</v>
       </c>
       <c r="P14">
-        <v>3.0951081467115327E-3</v>
+        <v>1.7225648005951964E-4</v>
       </c>
       <c r="Q14">
-        <v>3.2900605473727062E-3</v>
+        <v>-9.8433482570649631E-3</v>
       </c>
       <c r="R14">
-        <v>-4.4638124408031676E-5</v>
-      </c>
-      <c r="S14">
-        <v>2.7131022368467764E-3</v>
-      </c>
-      <c r="T14">
-        <v>-4.6980876883268106E-4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.45">
+        <v>3.3621391847473399E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B15">
-        <v>-0.10793004989242458</v>
+        <v>-1.0254622771733349E-2</v>
       </c>
       <c r="C15">
-        <v>1.4827892130014485E-4</v>
+        <v>-1.0836520001444264E-4</v>
       </c>
       <c r="D15">
-        <v>-1.7171163662585268E-4</v>
+        <v>2.0146364281990227E-5</v>
       </c>
       <c r="E15">
-        <v>1.5359142673637339E-6</v>
+        <v>-2.1259597245707897E-7</v>
       </c>
       <c r="F15">
-        <v>2.2592037170349449E-4</v>
+        <v>-1.0061650106994697E-4</v>
       </c>
       <c r="G15">
-        <v>1.2379578923736121E-3</v>
+        <v>-5.5516971335677908E-5</v>
       </c>
       <c r="H15">
-        <v>-1.6653665831099914E-3</v>
+        <v>4.5171837507327608E-4</v>
       </c>
       <c r="I15">
-        <v>-1.4460380100188514E-4</v>
+        <v>-1.2967331318152614E-5</v>
       </c>
       <c r="J15">
-        <v>5.1974690662834853E-5</v>
+        <v>-4.2537009316695543E-5</v>
       </c>
       <c r="K15">
-        <v>-2.0619608947031838E-4</v>
+        <v>-2.044245098543395E-4</v>
       </c>
       <c r="L15">
-        <v>-5.3155510186194484E-4</v>
+        <v>-4.7491405347423687E-5</v>
       </c>
       <c r="M15">
-        <v>-7.546836858702481E-5</v>
+        <v>-1.108460694897777E-4</v>
       </c>
       <c r="N15">
-        <v>3.0587759543058723E-3</v>
+        <v>2.1641988894057277E-5</v>
       </c>
       <c r="O15">
-        <v>3.0951081467115327E-3</v>
+        <v>1.7225648005951964E-4</v>
       </c>
       <c r="P15">
-        <v>7.0406869935320431E-3</v>
+        <v>8.9711565213435512E-5</v>
       </c>
       <c r="Q15">
-        <v>3.4106630666730893E-3</v>
+        <v>-3.207359265305753E-4</v>
       </c>
       <c r="R15">
-        <v>-3.630839127780137E-5</v>
-      </c>
-      <c r="S15">
-        <v>1.7739226137818266E-3</v>
-      </c>
-      <c r="T15">
-        <v>1.185415452868357E-3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.45">
+        <v>-1.8901917911212079E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B16">
-        <v>-1.4835959876128364E-2</v>
+        <v>0.53874062547355428</v>
       </c>
       <c r="C16">
-        <v>-9.5053186783118391E-5</v>
+        <v>-3.3466507370939758E-4</v>
       </c>
       <c r="D16">
-        <v>-2.6502242576178798E-4</v>
+        <v>1.3248957791701862E-3</v>
       </c>
       <c r="E16">
-        <v>2.438407671292133E-6</v>
+        <v>-1.396862500921772E-5</v>
       </c>
       <c r="F16">
-        <v>-2.4121382828014358E-4</v>
+        <v>1.1107556451979448E-2</v>
       </c>
       <c r="G16">
-        <v>4.4738993930741003E-4</v>
+        <v>8.8369813352681039E-3</v>
       </c>
       <c r="H16">
-        <v>-2.5592008068141183E-3</v>
+        <v>-1.2415343685808766E-3</v>
       </c>
       <c r="I16">
-        <v>-8.3485450364707879E-5</v>
+        <v>-1.8771328538540744E-3</v>
       </c>
       <c r="J16">
-        <v>-9.7095857401441809E-4</v>
+        <v>-5.0012867754745984E-4</v>
       </c>
       <c r="K16">
-        <v>-1.1966821541551983E-3</v>
+        <v>7.7797411614440037E-4</v>
       </c>
       <c r="L16">
-        <v>-1.3963484469953419E-3</v>
+        <v>-2.3568185003525477E-3</v>
       </c>
       <c r="M16">
-        <v>1.82046751185376E-4</v>
+        <v>1.042019450191789E-2</v>
       </c>
       <c r="N16">
-        <v>3.2389422085004355E-3</v>
+        <v>-1.0732736406725899E-2</v>
       </c>
       <c r="O16">
-        <v>3.2900605473727062E-3</v>
+        <v>-9.8433482570649631E-3</v>
       </c>
       <c r="P16">
-        <v>3.4106630666730893E-3</v>
+        <v>-3.207359265305753E-4</v>
       </c>
       <c r="Q16">
-        <v>6.5669970986562522E-3</v>
+        <v>2.9530938273033908E-2</v>
       </c>
       <c r="R16">
-        <v>5.2417268486885471E-5</v>
-      </c>
-      <c r="S16">
-        <v>2.408071300868096E-5</v>
-      </c>
-      <c r="T16">
-        <v>3.2451092601432402E-3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.45">
+        <v>-2.8884876664336735E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B17">
-        <v>-1.9921962809700509E-2</v>
+        <v>-3.973096889765916</v>
       </c>
       <c r="C17">
-        <v>-7.7364248326043373E-6</v>
+        <v>4.7173049938376722E-3</v>
       </c>
       <c r="D17">
-        <v>-8.9100406146334498E-6</v>
+        <v>-9.6179073198524243E-3</v>
       </c>
       <c r="E17">
-        <v>4.0657622425960691E-8</v>
+        <v>1.019425455645008E-4</v>
       </c>
       <c r="F17">
-        <v>-1.8265244248629289E-4</v>
+        <v>-1.0361329999183677E-2</v>
       </c>
       <c r="G17">
-        <v>-1.2569327006975626E-4</v>
+        <v>-8.1509555860503971E-3</v>
       </c>
       <c r="H17">
-        <v>-2.0138015442662744E-4</v>
+        <v>-4.3199896539518431E-2</v>
       </c>
       <c r="I17">
-        <v>1.1475949648633461E-4</v>
+        <v>9.5786317840187984E-4</v>
       </c>
       <c r="J17">
-        <v>-1.796116370937893E-4</v>
+        <v>-4.5658547075397883E-3</v>
       </c>
       <c r="K17">
-        <v>-1.9558995899237713E-4</v>
+        <v>2.1790331888380116E-3</v>
       </c>
       <c r="L17">
-        <v>-7.175216639173981E-5</v>
+        <v>-2.6313988096598809E-3</v>
       </c>
       <c r="M17">
-        <v>-5.8933168319049995E-5</v>
+        <v>-1.3117976257928422E-2</v>
       </c>
       <c r="N17">
-        <v>-1.342885853051428E-4</v>
+        <v>1.1057574606980491E-2</v>
       </c>
       <c r="O17">
-        <v>-4.4638124408031676E-5</v>
+        <v>3.3621391847473399E-3</v>
       </c>
       <c r="P17">
-        <v>-3.630839127780137E-5</v>
+        <v>-1.8901917911212079E-3</v>
       </c>
       <c r="Q17">
-        <v>5.2417268486885471E-5</v>
+        <v>-2.8884876664336735E-2</v>
       </c>
       <c r="R17">
-        <v>7.4359816795321995E-5</v>
-      </c>
-      <c r="S17">
-        <v>-2.5404293637631227E-4</v>
-      </c>
-      <c r="T17">
-        <v>-6.5750326306059125E-4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18">
-        <v>0.35725714638875988</v>
-      </c>
-      <c r="C18">
-        <v>-6.5627161746209279E-4</v>
-      </c>
-      <c r="D18">
-        <v>-2.7610964267736214E-4</v>
-      </c>
-      <c r="E18">
-        <v>2.809613806166921E-6</v>
-      </c>
-      <c r="F18">
-        <v>9.9638628181522083E-4</v>
-      </c>
-      <c r="G18">
-        <v>1.6293921218012769E-3</v>
-      </c>
-      <c r="H18">
-        <v>-2.2488595407094917E-3</v>
-      </c>
-      <c r="I18">
-        <v>-1.2760094487212347E-3</v>
-      </c>
-      <c r="J18">
-        <v>7.701805963137155E-4</v>
-      </c>
-      <c r="K18">
-        <v>4.1501640030809249E-4</v>
-      </c>
-      <c r="L18">
-        <v>9.0241584827686992E-4</v>
-      </c>
-      <c r="M18">
-        <v>2.0450145324684473E-4</v>
-      </c>
-      <c r="N18">
-        <v>8.6147130719185197E-4</v>
-      </c>
-      <c r="O18">
-        <v>2.7131022368467764E-3</v>
-      </c>
-      <c r="P18">
-        <v>1.7739226137818266E-3</v>
-      </c>
-      <c r="Q18">
-        <v>2.408071300868096E-5</v>
-      </c>
-      <c r="R18">
-        <v>-2.5404293637631227E-4</v>
-      </c>
-      <c r="S18">
-        <v>9.7088365425418606E-3</v>
-      </c>
-      <c r="T18">
-        <v>8.0095189637951047E-3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19">
-        <v>-3.0024156185576474</v>
-      </c>
-      <c r="C19">
-        <v>-3.3823911252607811E-3</v>
-      </c>
-      <c r="D19">
-        <v>-4.0679282969788861E-3</v>
-      </c>
-      <c r="E19">
-        <v>4.1336281359242754E-5</v>
-      </c>
-      <c r="F19">
-        <v>-5.3423360247093279E-3</v>
-      </c>
-      <c r="G19">
-        <v>-3.364111670384847E-3</v>
-      </c>
-      <c r="H19">
-        <v>-2.3850308120631505E-2</v>
-      </c>
-      <c r="I19">
-        <v>-8.592742683163344E-3</v>
-      </c>
-      <c r="J19">
-        <v>-7.3773887527030114E-3</v>
-      </c>
-      <c r="K19">
-        <v>-1.241450547843256E-2</v>
-      </c>
-      <c r="L19">
-        <v>-1.0816096040140584E-2</v>
-      </c>
-      <c r="M19">
-        <v>-1.2345642577996694E-2</v>
-      </c>
-      <c r="N19">
-        <v>-5.4344618842005609E-4</v>
-      </c>
-      <c r="O19">
-        <v>-4.6980876883268106E-4</v>
-      </c>
-      <c r="P19">
-        <v>1.185415452868357E-3</v>
-      </c>
-      <c r="Q19">
-        <v>3.2451092601432402E-3</v>
-      </c>
-      <c r="R19">
-        <v>-6.5750326306059125E-4</v>
-      </c>
-      <c r="S19">
-        <v>8.0095189637951047E-3</v>
-      </c>
-      <c r="T19">
-        <v>0.12064604664263855</v>
+        <v>0.254431725689232</v>
       </c>
     </row>
   </sheetData>

</xml_diff>